<commit_message>
WP17/18-Auswertungen in Unterordner, Index/ ausgegliedert
- data/WP17_*.xlsx → data/WP17/, data/WP18_*.xlsx → data/WP18/
- index_parteien.xlsx + neue abgeordnete.xlsx in Index/
- .gitignore: R-Session-Dateien, index-Backups, WIP-Pfade
- R/laufzeiten-auswerten.R, landtag.py, SKILL.md aktualisiert
- auswertung_fehlende_daten.md entfernt (Punkte adressiert)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ALLE_topthemen_zeitreihe.xlsx
+++ b/data/ALLE_topthemen_zeitreihe.xlsx
@@ -2592,7 +2592,7 @@
         <v>12</v>
       </c>
       <c r="C58" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D58" t="s">
         <v>11</v>
@@ -4317,6 +4317,27 @@
       <c r="K107" t="n">
         <v>9</v>
       </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1"/>
+      <c r="B108" t="s">
+        <v>12</v>
+      </c>
+      <c r="C108" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" t="s">
+        <v>14</v>
+      </c>
+      <c r="E108" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108"/>
+      <c r="G108"/>
+      <c r="H108"/>
+      <c r="I108"/>
+      <c r="J108"/>
+      <c r="K108"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4552,13 +4573,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB289F36-5F58-4D7C-A84B-8FDE997C02CB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A7E6E0-7EB6-4FDA-BA71-6243DC891F32}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BE78630-9F48-4CDA-BD8B-8D202A00111C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FFD644B-CF65-495C-9936-1168FFDA2612}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FBBC2BD-D5F4-4E81-B351-E1D962B8320E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B82B68FF-A4B4-44DC-A165-1DC66D6B73D1}"/>
 </file>
</xml_diff>